<commit_message>
Extend job-titles Excel import to set institutional competency levels
Add 11 optional columns (one per real institutional competency) so a
required_level can be set for a job title during bulk import, closing
the gap where the import covered core fields but not competencies. A
blank cell leaves an existing assignment untouched.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/sru-job-titles-import-template.xlsx
+++ b/public/templates/sru-job-titles-import-template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="40">
   <si>
     <t>تعليمات استيراد المسميات الوظيفية</t>
   </si>
@@ -44,6 +44,21 @@
     <t>8. احذف صف المثال (الصف الثاني في ورقة "المسميات الوظيفية") قبل الاستيراد الفعلي إذا لم يكن بيانات حقيقية.</t>
   </si>
   <si>
+    <t>الجدارات المؤسسية (اختياري):</t>
+  </si>
+  <si>
+    <t>9. توجد 11 عمودًا إضافيًا اختياريًا، أحدها لكل جدارة مؤسسية (أعمدة G وما بعدها في ورقة "المسميات الوظيفية") — إذا ملأت خلية منها، ستُحدَّد مستوى تلك الجدارة لهذا المسمى الوظيفي.</t>
+  </si>
+  <si>
+    <t>10. القيم المقبولة لمستوى الجدارة: أساسي، ممارس، متقدم، محترف. أي خلية فارغة تُترك دون تغيير (لن تُحذف جدارة محددة مسبقًا).</t>
+  </si>
+  <si>
+    <t>11. مثال: إذا وضعت "متقدم" في عمود "التواصل الفعال" لصف مسمى وظيفي معين، سيُحدَّد مستوى "متقدم" لجدارة "التواصل الفعال" لهذا المسمى.</t>
+  </si>
+  <si>
+    <t>لتحديد أكثر من خيار ترقية لنفس المسمى (مثل محلل أعمال مساعد الذي قد يترقى إلى محلل أعمال أو محلل بيانات)، استخدم استيراد المسار الوظيفي المنفصل من صفحة "المسار الوظيفي" — أضف صفًا مستقلًا لكل خيار ترقية بنفس عمود "من" وقيمة مختلفة في عمود "إلى".</t>
+  </si>
+  <si>
     <t>اسم المسمى الوظيفي</t>
   </si>
   <si>
@@ -65,6 +80,39 @@
     <t>الوصف الوظيفي</t>
   </si>
   <si>
+    <t>إدارة المخاطر</t>
+  </si>
+  <si>
+    <t>إدارة المهام والمشاريع</t>
+  </si>
+  <si>
+    <t>الأداء المالي</t>
+  </si>
+  <si>
+    <t>الامتثال والالتزام</t>
+  </si>
+  <si>
+    <t>التعامل مع التقارير والبيانات</t>
+  </si>
+  <si>
+    <t>التعامل مع التقنية والتحول الرقمي</t>
+  </si>
+  <si>
+    <t>التواصل الفعال</t>
+  </si>
+  <si>
+    <t>المساهمة في تعزيز الصورة الذهنية للجامعة</t>
+  </si>
+  <si>
+    <t>المشاركة في المسؤولية المجتمعية والعمل التطوعي</t>
+  </si>
+  <si>
+    <t>خدمة العميل</t>
+  </si>
+  <si>
+    <t>روح الفريق</t>
+  </si>
+  <si>
     <t>مثال: أخصائي موارد بشرية</t>
   </si>
   <si>
@@ -81,6 +129,9 @@
   </si>
   <si>
     <t>يتولى شاغل الوظيفة تنفيذ المهام التخصصية المتعلقة بالموارد البشرية...</t>
+  </si>
+  <si>
+    <t>متقدم</t>
   </si>
 </sst>
 </file>
@@ -487,7 +538,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="90" customWidth="1"/>
@@ -543,6 +594,41 @@
         <v>9</v>
       </c>
     </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -551,7 +637,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -560,52 +646,119 @@
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="30" customWidth="1"/>
     <col min="7" max="7" width="45" customWidth="1"/>
+    <col min="8" max="18" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q1" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="R1" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="D2" s="5">
         <v>9</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>22</v>
+        <v>38</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="N2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="O2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="P2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="R2" s="5" t="s">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Extend job-titles Excel import to set institutional competency levels (#130)
Add 11 optional columns (one per real institutional competency) so a
required_level can be set for a job title during bulk import, closing
the gap where the import covered core fields but not competencies. A
blank cell leaves an existing assignment untouched.

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/sru-job-titles-import-template.xlsx
+++ b/public/templates/sru-job-titles-import-template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="40">
   <si>
     <t>تعليمات استيراد المسميات الوظيفية</t>
   </si>
@@ -44,6 +44,21 @@
     <t>8. احذف صف المثال (الصف الثاني في ورقة "المسميات الوظيفية") قبل الاستيراد الفعلي إذا لم يكن بيانات حقيقية.</t>
   </si>
   <si>
+    <t>الجدارات المؤسسية (اختياري):</t>
+  </si>
+  <si>
+    <t>9. توجد 11 عمودًا إضافيًا اختياريًا، أحدها لكل جدارة مؤسسية (أعمدة G وما بعدها في ورقة "المسميات الوظيفية") — إذا ملأت خلية منها، ستُحدَّد مستوى تلك الجدارة لهذا المسمى الوظيفي.</t>
+  </si>
+  <si>
+    <t>10. القيم المقبولة لمستوى الجدارة: أساسي، ممارس، متقدم، محترف. أي خلية فارغة تُترك دون تغيير (لن تُحذف جدارة محددة مسبقًا).</t>
+  </si>
+  <si>
+    <t>11. مثال: إذا وضعت "متقدم" في عمود "التواصل الفعال" لصف مسمى وظيفي معين، سيُحدَّد مستوى "متقدم" لجدارة "التواصل الفعال" لهذا المسمى.</t>
+  </si>
+  <si>
+    <t>لتحديد أكثر من خيار ترقية لنفس المسمى (مثل محلل أعمال مساعد الذي قد يترقى إلى محلل أعمال أو محلل بيانات)، استخدم استيراد المسار الوظيفي المنفصل من صفحة "المسار الوظيفي" — أضف صفًا مستقلًا لكل خيار ترقية بنفس عمود "من" وقيمة مختلفة في عمود "إلى".</t>
+  </si>
+  <si>
     <t>اسم المسمى الوظيفي</t>
   </si>
   <si>
@@ -65,6 +80,39 @@
     <t>الوصف الوظيفي</t>
   </si>
   <si>
+    <t>إدارة المخاطر</t>
+  </si>
+  <si>
+    <t>إدارة المهام والمشاريع</t>
+  </si>
+  <si>
+    <t>الأداء المالي</t>
+  </si>
+  <si>
+    <t>الامتثال والالتزام</t>
+  </si>
+  <si>
+    <t>التعامل مع التقارير والبيانات</t>
+  </si>
+  <si>
+    <t>التعامل مع التقنية والتحول الرقمي</t>
+  </si>
+  <si>
+    <t>التواصل الفعال</t>
+  </si>
+  <si>
+    <t>المساهمة في تعزيز الصورة الذهنية للجامعة</t>
+  </si>
+  <si>
+    <t>المشاركة في المسؤولية المجتمعية والعمل التطوعي</t>
+  </si>
+  <si>
+    <t>خدمة العميل</t>
+  </si>
+  <si>
+    <t>روح الفريق</t>
+  </si>
+  <si>
     <t>مثال: أخصائي موارد بشرية</t>
   </si>
   <si>
@@ -81,6 +129,9 @@
   </si>
   <si>
     <t>يتولى شاغل الوظيفة تنفيذ المهام التخصصية المتعلقة بالموارد البشرية...</t>
+  </si>
+  <si>
+    <t>متقدم</t>
   </si>
 </sst>
 </file>
@@ -487,7 +538,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="90" customWidth="1"/>
@@ -543,6 +594,41 @@
         <v>9</v>
       </c>
     </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -551,7 +637,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -560,52 +646,119 @@
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="30" customWidth="1"/>
     <col min="7" max="7" width="45" customWidth="1"/>
+    <col min="8" max="18" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q1" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="R1" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="D2" s="5">
         <v>9</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>22</v>
+        <v>38</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="N2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="O2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="P2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="R2" s="5" t="s">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>